<commit_message>
Timothy/Eclat recommendation is displayed on schedule
</commit_message>
<xml_diff>
--- a/data/recommended_staff_schedule.xlsx
+++ b/data/recommended_staff_schedule.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,12 +483,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>test</t>
+          <t>mike</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thusday </t>
+          <t>Friday</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -503,7 +503,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Bush - The Land of Milk and Honey Tour</t>
+          <t>Treaty Oak Revival - West Texas Degenerate Tour</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -526,7 +526,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Manager</t>
+          <t>eployee</t>
         </is>
       </c>
     </row>
@@ -538,22 +538,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Thusday </t>
+          <t>Saturday</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>19:00:00</t>
+          <t>19:30:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>19:00:00</t>
+          <t>19:30:00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bush - The Land of Milk and Honey Tour</t>
+          <t>Charlie Puth: Whatever's Clever! World Tour</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -575,206 +575,6 @@
         <v>0.3</v>
       </c>
       <c r="J3" t="inlineStr">
-        <is>
-          <t>eployee</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>19:00:00</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>19:00:00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Treaty Oak Revival - West Texas Degenerate Tour</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>WAMU Theater</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Waji’s</t>
-        </is>
-      </c>
-      <c r="I4" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>mike</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Friday</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>19:00:00</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>19:00:00</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Treaty Oak Revival - West Texas Degenerate Tour</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>WAMU Theater</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Waji’s</t>
-        </is>
-      </c>
-      <c r="I5" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>eployee</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>test</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Saturday </t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>19:30:00</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>19:30:00</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Charlie Puth: Whatever's Clever! World Tour</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>WAMU Theater</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Waji’s</t>
-        </is>
-      </c>
-      <c r="I6" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Manager</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>mike</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Saturday </t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>19:30:00</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>19:30:00</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Charlie Puth: Whatever's Clever! World Tour</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>WAMU Theater</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Waji’s</t>
-        </is>
-      </c>
-      <c r="I7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="J7" t="inlineStr">
         <is>
           <t>eployee</t>
         </is>

</xml_diff>